<commit_message>
MEC Software Tracker - initial deploy
</commit_message>
<xml_diff>
--- a/public/ข้อมูลโปรแกรมทั้งหมด-07-11-2568.xlsx
+++ b/public/ข้อมูลโปรแกรมทั้งหมด-07-11-2568.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MECPatiwatM\Desktop\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MECPatiwatM\Desktop\Software-MEC\Software MEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933D14F0-FD66-4550-9720-0A65F2FD08FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7374C573-9C1E-4E27-ABE3-8C601BA813C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{D1DED1F2-854C-4734-8246-D589BEF0D1B1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D1DED1F2-854C-4734-8246-D589BEF0D1B1}"/>
   </bookViews>
   <sheets>
     <sheet name="รวมทุกโปรแกรม" sheetId="1" r:id="rId1"/>
@@ -3283,9 +3283,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;฿&quot;* #,##0.00_-;\-&quot;฿&quot;* #,##0.00_-;_-&quot;฿&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="187" formatCode="&quot;฿&quot;#,##0"/>
+    <numFmt numFmtId="188" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="32" x14ac:knownFonts="1">
     <font>
@@ -3868,7 +3869,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4023,9 +4024,6 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4035,14 +4033,8 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="1" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4051,9 +4043,6 @@
     <xf numFmtId="187" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4126,9 +4115,6 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="1" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4136,11 +4122,26 @@
     <xf numFmtId="187" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="187" fontId="0" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="15" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="187" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="188" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="188" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="10" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -4215,6 +4216,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="188" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -7963,6 +7967,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="8">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9B934A9D-5193-4E1B-809E-7987A96DA92C}">
+  <we:reference id="29673e3c-d826-4f00-92ee-162334a52b1a" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;ab223ec1-5d4c-4fe9-94e1-6d4b86d1afca&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0122E76-4570-4F52-8D43-4E366FEBC83C}">
   <dimension ref="A1:H28"/>
@@ -8000,7 +8026,7 @@
       <c r="G1" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="83" t="s">
+      <c r="H1" s="79" t="s">
         <v>7</v>
       </c>
     </row>
@@ -8014,662 +8040,662 @@
       <c r="C2" s="65">
         <v>10</v>
       </c>
-      <c r="D2" s="66">
-        <v>244409</v>
-      </c>
-      <c r="E2" s="67" t="s">
+      <c r="D2" s="114">
+        <v>46082</v>
+      </c>
+      <c r="E2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="68">
+      <c r="F2" s="67">
         <v>9600</v>
       </c>
-      <c r="G2" s="85">
+      <c r="G2" s="81">
         <v>96000</v>
       </c>
-      <c r="H2" s="84">
+      <c r="H2" s="80">
         <f>G2/12*10</f>
         <v>80000</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="74">
+      <c r="C3" s="72">
         <v>20</v>
       </c>
-      <c r="D3" s="75">
-        <v>25373</v>
-      </c>
-      <c r="E3" s="76" t="s">
+      <c r="D3" s="115">
+        <v>46192</v>
+      </c>
+      <c r="E3" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="77">
+      <c r="F3" s="74">
         <v>13800</v>
       </c>
-      <c r="G3" s="86">
+      <c r="G3" s="82">
         <v>276000</v>
       </c>
-      <c r="H3" s="84">
+      <c r="H3" s="80">
         <f>G3/12*6</f>
         <v>138000</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A4" s="69"/>
-      <c r="B4" s="78" t="s">
+      <c r="A4" s="68"/>
+      <c r="B4" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="79">
+      <c r="C4" s="76">
         <v>10</v>
       </c>
-      <c r="D4" s="80">
-        <v>26117</v>
-      </c>
-      <c r="E4" s="81" t="s">
+      <c r="D4" s="116">
+        <v>46937</v>
+      </c>
+      <c r="E4" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="82">
+      <c r="F4" s="78">
         <v>41400</v>
       </c>
-      <c r="G4" s="87">
+      <c r="G4" s="83">
         <v>414000</v>
       </c>
-      <c r="H4" s="84"/>
+      <c r="H4" s="80"/>
     </row>
     <row r="5" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A5" s="69"/>
-      <c r="B5" s="73" t="s">
+      <c r="A5" s="68"/>
+      <c r="B5" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="74">
+      <c r="C5" s="72">
         <v>21</v>
       </c>
-      <c r="D5" s="75">
-        <v>25446</v>
-      </c>
-      <c r="E5" s="76" t="s">
+      <c r="D5" s="115">
+        <v>46265</v>
+      </c>
+      <c r="E5" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="77">
+      <c r="F5" s="74">
         <v>13800</v>
       </c>
-      <c r="G5" s="86">
+      <c r="G5" s="82">
         <f>F5*21</f>
         <v>289800</v>
       </c>
-      <c r="H5" s="84">
+      <c r="H5" s="80">
         <f>G5/12*4</f>
         <v>96600</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A6" s="69"/>
-      <c r="B6" s="73" t="s">
+      <c r="A6" s="68"/>
+      <c r="B6" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="74">
+      <c r="C6" s="72">
         <v>10</v>
       </c>
-      <c r="D6" s="75">
+      <c r="D6" s="115">
         <v>46383</v>
       </c>
-      <c r="E6" s="76" t="s">
+      <c r="E6" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="77">
+      <c r="F6" s="74">
         <v>13800</v>
       </c>
-      <c r="G6" s="86">
+      <c r="G6" s="82">
         <f>F6*10</f>
         <v>138000</v>
       </c>
-      <c r="H6" s="84">
+      <c r="H6" s="80">
         <f>G6/12*12</f>
         <v>138000</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A7" s="69"/>
-      <c r="B7" s="73" t="s">
+      <c r="A7" s="68"/>
+      <c r="B7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="74">
+      <c r="C7" s="72">
         <v>4</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="115">
         <v>46265</v>
       </c>
-      <c r="E7" s="76" t="s">
+      <c r="E7" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="77">
+      <c r="F7" s="74">
         <v>53000</v>
       </c>
-      <c r="G7" s="86">
+      <c r="G7" s="82">
         <v>212000</v>
       </c>
-      <c r="H7" s="84">
+      <c r="H7" s="80">
         <f>G7/12*4</f>
         <v>70666.666666666672</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A8" s="69"/>
-      <c r="B8" s="73" t="s">
+      <c r="A8" s="68"/>
+      <c r="B8" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="74">
+      <c r="C8" s="72">
         <v>3</v>
       </c>
-      <c r="D8" s="75">
+      <c r="D8" s="115">
         <v>46206</v>
       </c>
-      <c r="E8" s="76" t="s">
+      <c r="E8" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="77">
+      <c r="F8" s="74">
         <v>53000</v>
       </c>
-      <c r="G8" s="86">
+      <c r="G8" s="82">
         <v>159000</v>
       </c>
-      <c r="H8" s="84">
+      <c r="H8" s="80">
         <f>G8/12*6</f>
         <v>79500</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A9" s="69"/>
-      <c r="B9" s="73" t="s">
+      <c r="A9" s="68"/>
+      <c r="B9" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="74">
+      <c r="C9" s="72">
         <v>5</v>
       </c>
-      <c r="D9" s="75">
+      <c r="D9" s="115">
         <v>46186</v>
       </c>
-      <c r="E9" s="76" t="s">
+      <c r="E9" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="77">
+      <c r="F9" s="74">
         <v>20000</v>
       </c>
-      <c r="G9" s="86">
+      <c r="G9" s="82">
         <v>100000</v>
       </c>
-      <c r="H9" s="84">
+      <c r="H9" s="80">
         <f>G9/12*6</f>
         <v>50000</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A10" s="69"/>
-      <c r="B10" s="73" t="s">
+      <c r="A10" s="68"/>
+      <c r="B10" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="74">
+      <c r="C10" s="72">
         <v>6</v>
       </c>
-      <c r="D10" s="75">
+      <c r="D10" s="115">
         <v>46356</v>
       </c>
-      <c r="E10" s="76" t="s">
+      <c r="E10" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="77">
+      <c r="F10" s="74">
         <v>75000</v>
       </c>
-      <c r="G10" s="86">
+      <c r="G10" s="82">
         <v>450000</v>
       </c>
-      <c r="H10" s="84">
+      <c r="H10" s="80">
         <f>G10/12*1</f>
         <v>37500</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A11" s="69"/>
-      <c r="B11" s="73" t="s">
+      <c r="A11" s="68"/>
+      <c r="B11" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="74">
+      <c r="C11" s="72">
         <v>1</v>
       </c>
-      <c r="D11" s="75">
+      <c r="D11" s="115">
         <v>46409</v>
       </c>
-      <c r="E11" s="76" t="s">
+      <c r="E11" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="77">
+      <c r="F11" s="74">
         <v>78500</v>
       </c>
-      <c r="G11" s="86">
+      <c r="G11" s="82">
         <v>78500</v>
       </c>
-      <c r="H11" s="84"/>
+      <c r="H11" s="80"/>
     </row>
     <row r="12" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A12" s="69"/>
-      <c r="B12" s="73" t="s">
+      <c r="A12" s="68"/>
+      <c r="B12" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="74">
+      <c r="C12" s="72">
         <v>6</v>
       </c>
-      <c r="D12" s="75">
+      <c r="D12" s="115">
         <v>46356</v>
       </c>
-      <c r="E12" s="76" t="s">
+      <c r="E12" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="77">
+      <c r="F12" s="74">
         <v>11000</v>
       </c>
-      <c r="G12" s="86">
+      <c r="G12" s="82">
         <v>66000</v>
       </c>
-      <c r="H12" s="84">
+      <c r="H12" s="80">
         <f>G12/12*1</f>
         <v>5500</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A13" s="69" t="s">
+      <c r="A13" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="70" t="s">
+      <c r="B13" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="71">
+      <c r="C13" s="70">
         <v>10</v>
       </c>
-      <c r="D13" s="72">
+      <c r="D13" s="117">
         <v>46280</v>
       </c>
-      <c r="E13" s="67" t="s">
+      <c r="E13" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="68">
+      <c r="F13" s="67">
         <v>930</v>
       </c>
-      <c r="G13" s="85">
+      <c r="G13" s="81">
         <v>9300</v>
       </c>
-      <c r="H13" s="84">
+      <c r="H13" s="80">
         <f>G13/12*3</f>
         <v>2325</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A14" s="69"/>
-      <c r="B14" s="70" t="s">
+      <c r="A14" s="68"/>
+      <c r="B14" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="71">
+      <c r="C14" s="70">
         <v>96</v>
       </c>
-      <c r="D14" s="72">
+      <c r="D14" s="117">
         <v>46409</v>
       </c>
-      <c r="E14" s="67" t="s">
+      <c r="E14" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="68">
+      <c r="F14" s="67">
         <v>2940</v>
       </c>
-      <c r="G14" s="85">
+      <c r="G14" s="81">
         <v>282240</v>
       </c>
-      <c r="H14" s="84">
+      <c r="H14" s="80">
         <f>G14/12*11</f>
         <v>258720</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A15" s="69"/>
-      <c r="B15" s="70" t="s">
+      <c r="A15" s="68"/>
+      <c r="B15" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="71">
+      <c r="C15" s="70">
         <v>50</v>
       </c>
-      <c r="D15" s="72">
+      <c r="D15" s="117">
         <v>46280</v>
       </c>
-      <c r="E15" s="67" t="s">
+      <c r="E15" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="68">
+      <c r="F15" s="67">
         <v>3100</v>
       </c>
-      <c r="G15" s="85">
+      <c r="G15" s="81">
         <v>155000</v>
       </c>
-      <c r="H15" s="84">
+      <c r="H15" s="80">
         <f>G15/12*3</f>
         <v>38750</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A16" s="69"/>
-      <c r="B16" s="70" t="s">
+      <c r="A16" s="68"/>
+      <c r="B16" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="71">
+      <c r="C16" s="70">
         <v>10</v>
       </c>
-      <c r="D16" s="72">
+      <c r="D16" s="117">
         <v>46409</v>
       </c>
-      <c r="E16" s="67" t="s">
+      <c r="E16" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="68">
+      <c r="F16" s="67">
         <v>6170</v>
       </c>
-      <c r="G16" s="85">
+      <c r="G16" s="81">
         <v>61700</v>
       </c>
-      <c r="H16" s="84">
+      <c r="H16" s="80">
         <f>G16/12*11</f>
         <v>56558.333333333336</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A17" s="69"/>
-      <c r="B17" s="70" t="s">
+      <c r="A17" s="68"/>
+      <c r="B17" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="71">
+      <c r="C17" s="70">
         <v>2</v>
       </c>
-      <c r="D17" s="72">
+      <c r="D17" s="117">
         <v>46128</v>
       </c>
-      <c r="E17" s="67" t="s">
+      <c r="E17" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="68">
+      <c r="F17" s="67">
         <v>12000</v>
       </c>
-      <c r="G17" s="85">
+      <c r="G17" s="81">
         <f>F17*C17</f>
         <v>24000</v>
       </c>
-      <c r="H17" s="84">
+      <c r="H17" s="80">
         <f>G17/12*8</f>
         <v>16000</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="70" t="s">
+      <c r="B18" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="71">
+      <c r="C18" s="70">
         <v>2</v>
       </c>
-      <c r="D18" s="72">
+      <c r="D18" s="117">
         <v>46203</v>
       </c>
-      <c r="E18" s="67" t="s">
+      <c r="E18" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="68">
+      <c r="F18" s="67">
         <v>63000</v>
       </c>
-      <c r="G18" s="85">
+      <c r="G18" s="81">
         <v>126000</v>
       </c>
-      <c r="H18" s="84">
+      <c r="H18" s="80">
         <f>G18/12*6</f>
         <v>63000</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A19" s="69" t="s">
+      <c r="A19" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="70" t="s">
+      <c r="B19" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="71">
+      <c r="C19" s="70">
         <v>70</v>
       </c>
-      <c r="D19" s="72">
+      <c r="D19" s="117">
         <v>46279</v>
       </c>
-      <c r="E19" s="67" t="s">
+      <c r="E19" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="68">
+      <c r="F19" s="67">
         <v>500</v>
       </c>
-      <c r="G19" s="85">
+      <c r="G19" s="81">
         <v>35000</v>
       </c>
-      <c r="H19" s="84"/>
+      <c r="H19" s="80"/>
     </row>
     <row r="20" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A20" s="69"/>
-      <c r="B20" s="70" t="s">
+      <c r="A20" s="68"/>
+      <c r="B20" s="69" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="71">
+      <c r="C20" s="70">
         <v>80</v>
       </c>
-      <c r="D20" s="72">
+      <c r="D20" s="117">
         <v>46279</v>
       </c>
-      <c r="E20" s="67" t="s">
+      <c r="E20" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="68">
+      <c r="F20" s="67">
         <v>750</v>
       </c>
-      <c r="G20" s="85">
+      <c r="G20" s="81">
         <v>60000</v>
       </c>
-      <c r="H20" s="84">
+      <c r="H20" s="80">
         <f>G20/12*3</f>
         <v>15000</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A21" s="69" t="s">
+      <c r="A21" s="68" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="70" t="s">
+      <c r="B21" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="71">
+      <c r="C21" s="70">
         <v>10</v>
       </c>
-      <c r="D21" s="72">
-        <v>25320</v>
-      </c>
-      <c r="E21" s="67" t="s">
+      <c r="D21" s="117">
+        <v>46139</v>
+      </c>
+      <c r="E21" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="F21" s="68">
+      <c r="F21" s="67">
         <v>12400</v>
       </c>
-      <c r="G21" s="85">
+      <c r="G21" s="81">
         <v>124000</v>
       </c>
-      <c r="H21" s="84">
+      <c r="H21" s="80">
         <f>G21/12*8</f>
         <v>82666.666666666672</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A22" s="69" t="s">
+      <c r="A22" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="70" t="s">
+      <c r="B22" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="71">
+      <c r="C22" s="70">
         <v>1</v>
       </c>
-      <c r="D22" s="72">
-        <v>25305</v>
-      </c>
-      <c r="E22" s="67" t="s">
+      <c r="D22" s="117">
+        <v>46124</v>
+      </c>
+      <c r="E22" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="68">
+      <c r="F22" s="67">
         <v>6600</v>
       </c>
-      <c r="G22" s="85">
+      <c r="G22" s="81">
         <v>6600</v>
       </c>
-      <c r="H22" s="84">
+      <c r="H22" s="80">
         <f>G22/12*8</f>
         <v>4400</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A23" s="69"/>
-      <c r="B23" s="70" t="s">
+      <c r="A23" s="68"/>
+      <c r="B23" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="71">
+      <c r="C23" s="70">
         <v>1</v>
       </c>
-      <c r="D23" s="72">
-        <v>25234</v>
-      </c>
-      <c r="E23" s="67" t="s">
+      <c r="D23" s="117">
+        <v>46053</v>
+      </c>
+      <c r="E23" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="68">
+      <c r="F23" s="67">
         <v>204000</v>
       </c>
-      <c r="G23" s="85">
+      <c r="G23" s="81">
         <v>204000</v>
       </c>
-      <c r="H23" s="84">
+      <c r="H23" s="80">
         <f>G23/12*11</f>
         <v>187000</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A24" s="69" t="s">
+      <c r="A24" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="70" t="s">
+      <c r="B24" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="C24" s="71">
+      <c r="C24" s="70">
         <v>1</v>
       </c>
-      <c r="D24" s="72">
-        <v>244560</v>
-      </c>
-      <c r="E24" s="67" t="s">
+      <c r="D24" s="117">
+        <v>46233</v>
+      </c>
+      <c r="E24" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="F24" s="68">
+      <c r="F24" s="67">
         <v>45000</v>
       </c>
-      <c r="G24" s="85">
+      <c r="G24" s="81">
         <v>45000</v>
       </c>
-      <c r="H24" s="84">
+      <c r="H24" s="80">
         <f>G24/12*5</f>
         <v>18750</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A25" s="69" t="s">
+      <c r="A25" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="70" t="s">
+      <c r="B25" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="71">
+      <c r="C25" s="70">
         <v>1</v>
       </c>
-      <c r="D25" s="72">
-        <v>25609</v>
-      </c>
-      <c r="E25" s="67" t="s">
+      <c r="D25" s="117">
+        <v>46428</v>
+      </c>
+      <c r="E25" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="68">
+      <c r="F25" s="67">
         <v>2000</v>
       </c>
-      <c r="G25" s="85">
+      <c r="G25" s="81">
         <v>2000</v>
       </c>
-      <c r="H25" s="84">
+      <c r="H25" s="80">
         <f>G25/12*10</f>
         <v>1666.6666666666665</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A26" s="108" t="s">
+      <c r="A26" s="104" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="109" t="s">
+      <c r="B26" s="105" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="110">
+      <c r="C26" s="106">
         <v>1</v>
       </c>
-      <c r="D26" s="111">
-        <v>25419</v>
-      </c>
-      <c r="E26" s="112" t="s">
+      <c r="D26" s="118">
+        <v>46238</v>
+      </c>
+      <c r="E26" s="107" t="s">
         <v>49</v>
       </c>
-      <c r="F26" s="113">
+      <c r="F26" s="108">
         <v>2000</v>
       </c>
-      <c r="G26" s="114">
+      <c r="G26" s="109">
         <v>2000</v>
       </c>
-      <c r="H26" s="115">
+      <c r="H26" s="110">
         <f>G26/12*4</f>
         <v>666.66666666666663</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="1" customFormat="1" ht="25.8" x14ac:dyDescent="0.65">
-      <c r="A27" s="116" t="s">
+      <c r="A27" s="111" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="116" t="s">
+      <c r="B27" s="111" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="76">
+      <c r="C27" s="73">
         <v>1</v>
       </c>
-      <c r="D27" s="117">
+      <c r="D27" s="119">
         <v>46038</v>
       </c>
-      <c r="E27" s="76" t="s">
+      <c r="E27" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="F27" s="118">
+      <c r="F27" s="112">
         <v>20800</v>
       </c>
-      <c r="G27" s="118">
+      <c r="G27" s="112">
         <v>20800</v>
       </c>
-      <c r="H27" s="118"/>
+      <c r="H27" s="112"/>
     </row>
     <row r="28" spans="1:8" s="1" customFormat="1" ht="25.8" x14ac:dyDescent="0.65">
       <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
+      <c r="D28" s="145"/>
       <c r="E28" s="5" t="s">
         <v>8</v>
       </c>
@@ -10934,7 +10960,7 @@
       <c r="F4" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="88" t="s">
+      <c r="G4" s="84" t="s">
         <v>98</v>
       </c>
       <c r="H4" s="6" t="s">
@@ -12111,8 +12137,8 @@
       <c r="B45" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="F45" s="90"/>
-      <c r="G45" s="90"/>
+      <c r="F45" s="86"/>
+      <c r="G45" s="86"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.8">
       <c r="A46" s="9">
@@ -12121,8 +12147,8 @@
       <c r="B46" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="F46" s="90"/>
-      <c r="G46" s="90"/>
+      <c r="F46" s="86"/>
+      <c r="G46" s="86"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.8">
       <c r="A48" s="132" t="s">
@@ -12938,7 +12964,7 @@
       <c r="F4" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="88" t="s">
+      <c r="G4" s="84" t="s">
         <v>98</v>
       </c>
       <c r="H4" s="6" t="s">
@@ -14286,7 +14312,7 @@
       <c r="A51" s="9">
         <v>48</v>
       </c>
-      <c r="B51" s="89" t="s">
+      <c r="B51" s="85" t="s">
         <v>328</v>
       </c>
       <c r="C51" s="6" t="s">
@@ -14297,7 +14323,7 @@
         <v>118</v>
       </c>
       <c r="F51" s="6"/>
-      <c r="G51" s="90" t="s">
+      <c r="G51" s="86" t="s">
         <v>330</v>
       </c>
       <c r="H51" s="6" t="s">
@@ -14685,75 +14711,75 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A66" s="91" t="s">
+      <c r="A66" s="87" t="s">
         <v>390</v>
       </c>
-      <c r="B66" s="91"/>
+      <c r="B66" s="87"/>
     </row>
     <row r="67" spans="1:9" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A67" s="92">
+      <c r="A67" s="88">
         <v>1</v>
       </c>
-      <c r="B67" s="91"/>
-      <c r="C67" s="91" t="s">
+      <c r="B67" s="87"/>
+      <c r="C67" s="87" t="s">
         <v>391</v>
       </c>
-      <c r="D67" s="91" t="s">
+      <c r="D67" s="87" t="s">
         <v>392</v>
       </c>
-      <c r="E67" s="91" t="s">
+      <c r="E67" s="87" t="s">
         <v>393</v>
       </c>
-      <c r="F67" s="91"/>
-      <c r="G67" s="91"/>
-      <c r="H67" s="91"/>
-      <c r="I67" s="91" t="s">
+      <c r="F67" s="87"/>
+      <c r="G67" s="87"/>
+      <c r="H67" s="87"/>
+      <c r="I67" s="87" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A68" s="92">
+      <c r="A68" s="88">
         <v>2</v>
       </c>
-      <c r="B68" s="91" t="s">
+      <c r="B68" s="87" t="s">
         <v>394</v>
       </c>
-      <c r="C68" s="91" t="s">
+      <c r="C68" s="87" t="s">
         <v>395</v>
       </c>
-      <c r="D68" s="91" t="s">
+      <c r="D68" s="87" t="s">
         <v>396</v>
       </c>
-      <c r="E68" s="93" t="s">
+      <c r="E68" s="89" t="s">
         <v>96</v>
       </c>
-      <c r="F68" s="91"/>
-      <c r="G68" s="91"/>
-      <c r="H68" s="91"/>
-      <c r="I68" s="91" t="s">
+      <c r="F68" s="87"/>
+      <c r="G68" s="87"/>
+      <c r="H68" s="87"/>
+      <c r="I68" s="87" t="s">
         <v>397</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A69" s="92">
+      <c r="A69" s="88">
         <v>3</v>
       </c>
-      <c r="B69" s="91" t="s">
+      <c r="B69" s="87" t="s">
         <v>299</v>
       </c>
-      <c r="C69" s="91" t="s">
+      <c r="C69" s="87" t="s">
         <v>398</v>
       </c>
-      <c r="D69" s="91" t="s">
+      <c r="D69" s="87" t="s">
         <v>399</v>
       </c>
-      <c r="E69" s="91" t="s">
+      <c r="E69" s="87" t="s">
         <v>400</v>
       </c>
-      <c r="F69" s="91"/>
-      <c r="G69" s="91"/>
-      <c r="H69" s="91"/>
-      <c r="I69" s="94" t="s">
+      <c r="F69" s="87"/>
+      <c r="G69" s="87"/>
+      <c r="H69" s="87"/>
+      <c r="I69" s="90" t="s">
         <v>274</v>
       </c>
     </row>
@@ -15929,7 +15955,7 @@
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
-      <c r="D8" s="95"/>
+      <c r="D8" s="91"/>
       <c r="E8" s="16"/>
       <c r="F8" s="52"/>
       <c r="G8" s="52"/>
@@ -16615,7 +16641,7 @@
       <c r="H3" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="105" t="s">
+      <c r="I3" s="101" t="s">
         <v>494</v>
       </c>
     </row>
@@ -16635,10 +16661,10 @@
       <c r="E4" s="16" t="s">
         <v>496</v>
       </c>
-      <c r="F4" s="104" t="s">
+      <c r="F4" s="100" t="s">
         <v>283</v>
       </c>
-      <c r="G4" s="104" t="s">
+      <c r="G4" s="100" t="s">
         <v>283</v>
       </c>
       <c r="H4" s="16" t="s">
@@ -16664,10 +16690,10 @@
       <c r="E5" s="16" t="s">
         <v>499</v>
       </c>
-      <c r="F5" s="104" t="s">
+      <c r="F5" s="100" t="s">
         <v>288</v>
       </c>
-      <c r="G5" s="104" t="s">
+      <c r="G5" s="100" t="s">
         <v>288</v>
       </c>
       <c r="H5" s="16" t="s">
@@ -16681,15 +16707,15 @@
       <c r="A6" s="15">
         <v>3</v>
       </c>
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="113" t="s">
         <v>501</v>
       </c>
-      <c r="C6" s="106"/>
-      <c r="D6" s="106"/>
-      <c r="E6" s="106"/>
-      <c r="F6" s="106"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="106" t="s">
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="103"/>
+      <c r="H6" s="102" t="s">
         <v>502</v>
       </c>
       <c r="I6" s="5"/>
@@ -16698,7 +16724,7 @@
       <c r="A7" s="15">
         <v>4</v>
       </c>
-      <c r="B7" s="119" t="s">
+      <c r="B7" s="113" t="s">
         <v>503</v>
       </c>
       <c r="C7" s="16"/>
@@ -16717,7 +16743,7 @@
       <c r="A8" s="15">
         <v>5</v>
       </c>
-      <c r="B8" s="119" t="s">
+      <c r="B8" s="113" t="s">
         <v>505</v>
       </c>
       <c r="C8" s="16"/>
@@ -17076,13 +17102,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="A26:B26"/>
@@ -17091,11 +17115,13 @@
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C28:D28"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:G3 C4:G12 H3:H12">
     <cfRule type="dataBar" priority="13">
@@ -17744,11 +17770,11 @@
       <c r="B3" s="27" t="s">
         <v>554</v>
       </c>
-      <c r="C3" s="98" t="str" cm="1">
+      <c r="C3" s="94" t="str" cm="1">
         <f t="array" ref="C3">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Aiyanat</v>
       </c>
-      <c r="D3" s="98" t="s">
+      <c r="D3" s="94" t="s">
         <v>555</v>
       </c>
       <c r="E3" s="27" t="s">
@@ -17768,11 +17794,11 @@
       <c r="B4" s="27" t="s">
         <v>558</v>
       </c>
-      <c r="C4" s="98" t="str" cm="1">
+      <c r="C4" s="94" t="str" cm="1">
         <f t="array" ref="C4">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Angkana</v>
       </c>
-      <c r="D4" s="98" t="s">
+      <c r="D4" s="94" t="s">
         <v>559</v>
       </c>
       <c r="E4" s="27" t="s">
@@ -17792,11 +17818,11 @@
       <c r="B5" s="27" t="s">
         <v>562</v>
       </c>
-      <c r="C5" s="98" t="str" cm="1">
+      <c r="C5" s="94" t="str" cm="1">
         <f t="array" ref="C5">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Anurak</v>
       </c>
-      <c r="D5" s="98" t="s">
+      <c r="D5" s="94" t="s">
         <v>563</v>
       </c>
       <c r="E5" s="27" t="s">
@@ -17813,7 +17839,7 @@
       <c r="A6" s="31">
         <v>4</v>
       </c>
-      <c r="B6" s="96" t="s">
+      <c r="B6" s="92" t="s">
         <v>566</v>
       </c>
       <c r="C6" s="44" t="str" cm="1">
@@ -17823,13 +17849,13 @@
       <c r="D6" s="44" t="s">
         <v>567</v>
       </c>
-      <c r="E6" s="97" t="s">
+      <c r="E6" s="93" t="s">
         <v>98</v>
       </c>
-      <c r="F6" s="96" t="s">
+      <c r="F6" s="92" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="96" t="s">
+      <c r="G6" s="92" t="s">
         <v>100</v>
       </c>
     </row>
@@ -17840,11 +17866,11 @@
       <c r="B7" s="27" t="s">
         <v>568</v>
       </c>
-      <c r="C7" s="98" t="str" cm="1">
+      <c r="C7" s="94" t="str" cm="1">
         <f t="array" ref="C7">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Apipong</v>
       </c>
-      <c r="D7" s="98" t="s">
+      <c r="D7" s="94" t="s">
         <v>569</v>
       </c>
       <c r="E7" s="27" t="s">
@@ -17864,11 +17890,11 @@
       <c r="B8" s="27" t="s">
         <v>572</v>
       </c>
-      <c r="C8" s="98" t="str" cm="1">
+      <c r="C8" s="94" t="str" cm="1">
         <f t="array" ref="C8">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Arnut</v>
       </c>
-      <c r="D8" s="98" t="s">
+      <c r="D8" s="94" t="s">
         <v>573</v>
       </c>
       <c r="E8" s="27" t="s">
@@ -17888,11 +17914,11 @@
       <c r="B9" s="27" t="s">
         <v>574</v>
       </c>
-      <c r="C9" s="98" t="str" cm="1">
+      <c r="C9" s="94" t="str" cm="1">
         <f t="array" ref="C9">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Benjamat</v>
       </c>
-      <c r="D9" s="98" t="s">
+      <c r="D9" s="94" t="s">
         <v>575</v>
       </c>
       <c r="E9" s="27" t="s">
@@ -17912,11 +17938,11 @@
       <c r="B10" s="27" t="s">
         <v>578</v>
       </c>
-      <c r="C10" s="98" t="str" cm="1">
+      <c r="C10" s="94" t="str" cm="1">
         <f t="array" ref="C10">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Bhusayamast</v>
       </c>
-      <c r="D10" s="98" t="s">
+      <c r="D10" s="94" t="s">
         <v>579</v>
       </c>
       <c r="E10" s="27" t="s">
@@ -17936,11 +17962,11 @@
       <c r="B11" s="27" t="s">
         <v>582</v>
       </c>
-      <c r="C11" s="98" t="str" cm="1">
+      <c r="C11" s="94" t="str" cm="1">
         <f t="array" ref="C11">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Chaiwat</v>
       </c>
-      <c r="D11" s="98" t="s">
+      <c r="D11" s="94" t="s">
         <v>583</v>
       </c>
       <c r="E11" s="27" t="s">
@@ -17957,17 +17983,17 @@
       <c r="A12" s="31">
         <v>10</v>
       </c>
-      <c r="B12" s="99" t="s">
+      <c r="B12" s="95" t="s">
         <v>585</v>
       </c>
-      <c r="C12" s="98" t="str" cm="1">
+      <c r="C12" s="94" t="str" cm="1">
         <f t="array" ref="C12">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Chalita</v>
       </c>
-      <c r="D12" s="98" t="s">
+      <c r="D12" s="94" t="s">
         <v>586</v>
       </c>
-      <c r="E12" s="100" t="s">
+      <c r="E12" s="96" t="s">
         <v>587</v>
       </c>
       <c r="F12" s="42" t="s">
@@ -17984,20 +18010,20 @@
       <c r="B13" s="27" t="s">
         <v>589</v>
       </c>
-      <c r="C13" s="98" t="str" cm="1">
+      <c r="C13" s="94" t="str" cm="1">
         <f t="array" ref="C13">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Chirawat</v>
       </c>
-      <c r="D13" s="98" t="s">
+      <c r="D13" s="94" t="s">
         <v>590</v>
       </c>
       <c r="E13" s="27" t="s">
         <v>309</v>
       </c>
-      <c r="F13" s="101" t="s">
+      <c r="F13" s="97" t="s">
         <v>591</v>
       </c>
-      <c r="G13" s="101" t="s">
+      <c r="G13" s="97" t="s">
         <v>592</v>
       </c>
     </row>
@@ -18008,11 +18034,11 @@
       <c r="B14" s="27" t="s">
         <v>593</v>
       </c>
-      <c r="C14" s="98" t="str" cm="1">
+      <c r="C14" s="94" t="str" cm="1">
         <f t="array" ref="C14">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Chissanupong</v>
       </c>
-      <c r="D14" s="98" t="s">
+      <c r="D14" s="94" t="s">
         <v>594</v>
       </c>
       <c r="E14" s="27" t="s">
@@ -18032,11 +18058,11 @@
       <c r="B15" s="27" t="s">
         <v>596</v>
       </c>
-      <c r="C15" s="98" t="str" cm="1">
+      <c r="C15" s="94" t="str" cm="1">
         <f t="array" ref="C15">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Damrongkiat</v>
       </c>
-      <c r="D15" s="98" t="s">
+      <c r="D15" s="94" t="s">
         <v>597</v>
       </c>
       <c r="E15" s="27" t="s">
@@ -18056,11 +18082,11 @@
       <c r="B16" s="27" t="s">
         <v>599</v>
       </c>
-      <c r="C16" s="98" t="str" cm="1">
+      <c r="C16" s="94" t="str" cm="1">
         <f t="array" ref="C16">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Decha</v>
       </c>
-      <c r="D16" s="98" t="s">
+      <c r="D16" s="94" t="s">
         <v>600</v>
       </c>
       <c r="E16" s="27" t="s">
@@ -18080,11 +18106,11 @@
       <c r="B17" s="27" t="s">
         <v>601</v>
       </c>
-      <c r="C17" s="98" t="str" cm="1">
+      <c r="C17" s="94" t="str" cm="1">
         <f t="array" ref="C17">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Detsakda</v>
       </c>
-      <c r="D17" s="98" t="s">
+      <c r="D17" s="94" t="s">
         <v>602</v>
       </c>
       <c r="E17" s="27" t="s">
@@ -18104,11 +18130,11 @@
       <c r="B18" s="27" t="s">
         <v>605</v>
       </c>
-      <c r="C18" s="98" t="str" cm="1">
+      <c r="C18" s="94" t="str" cm="1">
         <f t="array" ref="C18">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Ittidate</v>
       </c>
-      <c r="D18" s="98" t="s">
+      <c r="D18" s="94" t="s">
         <v>606</v>
       </c>
       <c r="E18" s="27" t="s">
@@ -18128,11 +18154,11 @@
       <c r="B19" s="27" t="s">
         <v>608</v>
       </c>
-      <c r="C19" s="98" t="str" cm="1">
+      <c r="C19" s="94" t="str" cm="1">
         <f t="array" ref="C19">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Jatupol</v>
       </c>
-      <c r="D19" s="98" t="s">
+      <c r="D19" s="94" t="s">
         <v>609</v>
       </c>
       <c r="E19" s="27" t="s">
@@ -18152,11 +18178,11 @@
       <c r="B20" s="27" t="s">
         <v>611</v>
       </c>
-      <c r="C20" s="98" t="str" cm="1">
+      <c r="C20" s="94" t="str" cm="1">
         <f t="array" ref="C20">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Jerapa</v>
       </c>
-      <c r="D20" s="98" t="s">
+      <c r="D20" s="94" t="s">
         <v>612</v>
       </c>
       <c r="E20" s="27" t="s">
@@ -18176,11 +18202,11 @@
       <c r="B21" s="27" t="s">
         <v>615</v>
       </c>
-      <c r="C21" s="98" t="str" cm="1">
+      <c r="C21" s="94" t="str" cm="1">
         <f t="array" ref="C21">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Jiraporn</v>
       </c>
-      <c r="D21" s="98" t="s">
+      <c r="D21" s="94" t="s">
         <v>616</v>
       </c>
       <c r="E21" s="27" t="s">
@@ -18200,11 +18226,11 @@
       <c r="B22" s="27" t="s">
         <v>619</v>
       </c>
-      <c r="C22" s="98" t="str" cm="1">
+      <c r="C22" s="94" t="str" cm="1">
         <f t="array" ref="C22">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanitta</v>
       </c>
-      <c r="D22" s="98" t="s">
+      <c r="D22" s="94" t="s">
         <v>620</v>
       </c>
       <c r="E22" s="27" t="s">
@@ -18224,11 +18250,11 @@
       <c r="B23" s="27" t="s">
         <v>623</v>
       </c>
-      <c r="C23" s="98" t="str" cm="1">
+      <c r="C23" s="94" t="str" cm="1">
         <f t="array" ref="C23">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanjanapha</v>
       </c>
-      <c r="D23" s="98" t="s">
+      <c r="D23" s="94" t="s">
         <v>624</v>
       </c>
       <c r="E23" s="27" t="s">
@@ -18246,11 +18272,11 @@
       <c r="B24" s="27" t="s">
         <v>626</v>
       </c>
-      <c r="C24" s="98" t="str" cm="1">
+      <c r="C24" s="94" t="str" cm="1">
         <f t="array" ref="C24">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanok</v>
       </c>
-      <c r="D24" s="98" t="s">
+      <c r="D24" s="94" t="s">
         <v>627</v>
       </c>
       <c r="E24" s="27" t="s">
@@ -18270,11 +18296,11 @@
       <c r="B25" s="27" t="s">
         <v>629</v>
       </c>
-      <c r="C25" s="98" t="str" cm="1">
+      <c r="C25" s="94" t="str" cm="1">
         <f t="array" ref="C25">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanokphon</v>
       </c>
-      <c r="D25" s="98" t="s">
+      <c r="D25" s="94" t="s">
         <v>630</v>
       </c>
       <c r="E25" s="27" t="s">
@@ -18294,8 +18320,8 @@
       <c r="B26" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="98"/>
-      <c r="D26" s="98"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
       <c r="E26" s="27"/>
       <c r="F26" s="27"/>
       <c r="G26" s="27"/>
@@ -18307,11 +18333,11 @@
       <c r="B27" s="27" t="s">
         <v>633</v>
       </c>
-      <c r="C27" s="98" t="str" cm="1">
+      <c r="C27" s="94" t="str" cm="1">
         <f t="array" ref="C27">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanraya</v>
       </c>
-      <c r="D27" s="98" t="s">
+      <c r="D27" s="94" t="s">
         <v>634</v>
       </c>
       <c r="E27" s="27" t="s">
@@ -18331,11 +18357,11 @@
       <c r="B28" s="27" t="s">
         <v>637</v>
       </c>
-      <c r="C28" s="98" t="str" cm="1">
+      <c r="C28" s="94" t="str" cm="1">
         <f t="array" ref="C28">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kanyapuk</v>
       </c>
-      <c r="D28" s="98" t="s">
+      <c r="D28" s="94" t="s">
         <v>638</v>
       </c>
       <c r="E28" s="27" t="s">
@@ -18355,11 +18381,11 @@
       <c r="B29" s="27" t="s">
         <v>640</v>
       </c>
-      <c r="C29" s="98" t="str" cm="1">
+      <c r="C29" s="94" t="str" cm="1">
         <f t="array" ref="C29">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Ketkanok</v>
       </c>
-      <c r="D29" s="98" t="s">
+      <c r="D29" s="94" t="s">
         <v>641</v>
       </c>
       <c r="E29" s="27" t="s">
@@ -18379,11 +18405,11 @@
       <c r="B30" s="27" t="s">
         <v>643</v>
       </c>
-      <c r="C30" s="98" t="str" cm="1">
+      <c r="C30" s="94" t="str" cm="1">
         <f t="array" ref="C30">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Khongsak</v>
       </c>
-      <c r="D30" s="98" t="s">
+      <c r="D30" s="94" t="s">
         <v>644</v>
       </c>
       <c r="E30" s="27" t="s">
@@ -18403,11 +18429,11 @@
       <c r="B31" s="27" t="s">
         <v>647</v>
       </c>
-      <c r="C31" s="98" t="str" cm="1">
+      <c r="C31" s="94" t="str" cm="1">
         <f t="array" ref="C31">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kiattisak</v>
       </c>
-      <c r="D31" s="98" t="s">
+      <c r="D31" s="94" t="s">
         <v>579</v>
       </c>
       <c r="E31" s="27" t="s">
@@ -18427,11 +18453,11 @@
       <c r="B32" s="27" t="s">
         <v>649</v>
       </c>
-      <c r="C32" s="98" t="str" cm="1">
+      <c r="C32" s="94" t="str" cm="1">
         <f t="array" ref="C32">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kingfai</v>
       </c>
-      <c r="D32" s="98" t="s">
+      <c r="D32" s="94" t="s">
         <v>650</v>
       </c>
       <c r="E32" s="27" t="s">
@@ -18451,11 +18477,11 @@
       <c r="B33" s="27" t="s">
         <v>652</v>
       </c>
-      <c r="C33" s="98" t="str" cm="1">
+      <c r="C33" s="94" t="str" cm="1">
         <f t="array" ref="C33">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kittipong</v>
       </c>
-      <c r="D33" s="98" t="s">
+      <c r="D33" s="94" t="s">
         <v>653</v>
       </c>
       <c r="E33" s="27" t="s">
@@ -18475,11 +18501,11 @@
       <c r="B34" s="27" t="s">
         <v>654</v>
       </c>
-      <c r="C34" s="98" t="str" cm="1">
+      <c r="C34" s="94" t="str" cm="1">
         <f t="array" ref="C34">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Korakot</v>
       </c>
-      <c r="D34" s="98" t="s">
+      <c r="D34" s="94" t="s">
         <v>655</v>
       </c>
       <c r="E34" s="27" t="s">
@@ -18499,11 +18525,11 @@
       <c r="B35" s="27" t="s">
         <v>657</v>
       </c>
-      <c r="C35" s="98" t="str" cm="1">
+      <c r="C35" s="94" t="str" cm="1">
         <f t="array" ref="C35">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kriangkai</v>
       </c>
-      <c r="D35" s="98" t="s">
+      <c r="D35" s="94" t="s">
         <v>658</v>
       </c>
       <c r="E35" s="27" t="s">
@@ -18523,11 +18549,11 @@
       <c r="B36" s="27" t="s">
         <v>659</v>
       </c>
-      <c r="C36" s="98" t="str" cm="1">
+      <c r="C36" s="94" t="str" cm="1">
         <f t="array" ref="C36">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kritsakorn</v>
       </c>
-      <c r="D36" s="98" t="s">
+      <c r="D36" s="94" t="s">
         <v>660</v>
       </c>
       <c r="E36" s="27" t="s">
@@ -18547,11 +18573,11 @@
       <c r="B37" s="27" t="s">
         <v>661</v>
       </c>
-      <c r="C37" s="98" t="str" cm="1">
+      <c r="C37" s="94" t="str" cm="1">
         <f t="array" ref="C37">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Krittapot</v>
       </c>
-      <c r="D37" s="98" t="s">
+      <c r="D37" s="94" t="s">
         <v>662</v>
       </c>
       <c r="E37" s="27" t="s">
@@ -18571,11 +18597,11 @@
       <c r="B38" s="27" t="s">
         <v>665</v>
       </c>
-      <c r="C38" s="98" t="str" cm="1">
+      <c r="C38" s="94" t="str" cm="1">
         <f t="array" ref="C38">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Kulthirath</v>
       </c>
-      <c r="D38" s="98" t="s">
+      <c r="D38" s="94" t="s">
         <v>666</v>
       </c>
       <c r="E38" s="27" t="s">
@@ -18595,14 +18621,14 @@
       <c r="B39" s="27" t="s">
         <v>669</v>
       </c>
-      <c r="C39" s="98" t="str" cm="1">
+      <c r="C39" s="94" t="str" cm="1">
         <f t="array" ref="C39">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Manlika</v>
       </c>
-      <c r="D39" s="98" t="s">
+      <c r="D39" s="94" t="s">
         <v>670</v>
       </c>
-      <c r="E39" s="102" t="s">
+      <c r="E39" s="98" t="s">
         <v>671</v>
       </c>
       <c r="F39" s="27" t="s">
@@ -18619,11 +18645,11 @@
       <c r="B40" s="27" t="s">
         <v>672</v>
       </c>
-      <c r="C40" s="98" t="str" cm="1">
+      <c r="C40" s="94" t="str" cm="1">
         <f t="array" ref="C40">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Marut</v>
       </c>
-      <c r="D40" s="98" t="s">
+      <c r="D40" s="94" t="s">
         <v>673</v>
       </c>
       <c r="E40" s="27" t="s">
@@ -18643,11 +18669,11 @@
       <c r="B41" s="27" t="s">
         <v>676</v>
       </c>
-      <c r="C41" s="98" t="str" cm="1">
+      <c r="C41" s="94" t="str" cm="1">
         <f t="array" ref="C41">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Mayuree</v>
       </c>
-      <c r="D41" s="98" t="s">
+      <c r="D41" s="94" t="s">
         <v>677</v>
       </c>
       <c r="E41" s="27" t="s">
@@ -18667,11 +18693,11 @@
       <c r="B42" s="27" t="s">
         <v>679</v>
       </c>
-      <c r="C42" s="98" t="str" cm="1">
+      <c r="C42" s="94" t="str" cm="1">
         <f t="array" ref="C42">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Metawee</v>
       </c>
-      <c r="D42" s="98" t="s">
+      <c r="D42" s="94" t="s">
         <v>680</v>
       </c>
       <c r="E42" s="27" t="s">
@@ -18691,11 +18717,11 @@
       <c r="B43" s="27" t="s">
         <v>683</v>
       </c>
-      <c r="C43" s="98" t="str" cm="1">
+      <c r="C43" s="94" t="str" cm="1">
         <f t="array" ref="C43">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nakaret</v>
       </c>
-      <c r="D43" s="98" t="s">
+      <c r="D43" s="94" t="s">
         <v>684</v>
       </c>
       <c r="E43" s="27" t="s">
@@ -18715,11 +18741,11 @@
       <c r="B44" s="27" t="s">
         <v>685</v>
       </c>
-      <c r="C44" s="98" t="str" cm="1">
+      <c r="C44" s="94" t="str" cm="1">
         <f t="array" ref="C44">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nanthaphon</v>
       </c>
-      <c r="D44" s="98" t="s">
+      <c r="D44" s="94" t="s">
         <v>686</v>
       </c>
       <c r="E44" s="27" t="s">
@@ -18739,11 +18765,11 @@
       <c r="B45" s="27" t="s">
         <v>688</v>
       </c>
-      <c r="C45" s="98" t="str" cm="1">
+      <c r="C45" s="94" t="str" cm="1">
         <f t="array" ref="C45">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nareenuch</v>
       </c>
-      <c r="D45" s="98" t="s">
+      <c r="D45" s="94" t="s">
         <v>689</v>
       </c>
       <c r="E45" s="27" t="s">
@@ -18763,11 +18789,11 @@
       <c r="B46" s="27" t="s">
         <v>691</v>
       </c>
-      <c r="C46" s="98" t="str" cm="1">
+      <c r="C46" s="94" t="str" cm="1">
         <f t="array" ref="C46">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Narisara</v>
       </c>
-      <c r="D46" s="98" t="s">
+      <c r="D46" s="94" t="s">
         <v>692</v>
       </c>
       <c r="E46" s="27" t="s">
@@ -18787,11 +18813,11 @@
       <c r="B47" s="27" t="s">
         <v>695</v>
       </c>
-      <c r="C47" s="98" t="str" cm="1">
+      <c r="C47" s="94" t="str" cm="1">
         <f t="array" ref="C47">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Natapong</v>
       </c>
-      <c r="D47" s="98" t="s">
+      <c r="D47" s="94" t="s">
         <v>696</v>
       </c>
       <c r="E47" s="27" t="s">
@@ -18811,11 +18837,11 @@
       <c r="B48" s="27" t="s">
         <v>698</v>
       </c>
-      <c r="C48" s="98" t="str" cm="1">
+      <c r="C48" s="94" t="str" cm="1">
         <f t="array" ref="C48">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattakorn</v>
       </c>
-      <c r="D48" s="98" t="s">
+      <c r="D48" s="94" t="s">
         <v>699</v>
       </c>
       <c r="E48" s="27" t="s">
@@ -18835,11 +18861,11 @@
       <c r="B49" s="27" t="s">
         <v>701</v>
       </c>
-      <c r="C49" s="98" t="str" cm="1">
+      <c r="C49" s="94" t="str" cm="1">
         <f t="array" ref="C49">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattaphon</v>
       </c>
-      <c r="D49" s="98" t="s">
+      <c r="D49" s="94" t="s">
         <v>702</v>
       </c>
       <c r="E49" s="27" t="s">
@@ -18859,11 +18885,11 @@
       <c r="B50" s="27" t="s">
         <v>703</v>
       </c>
-      <c r="C50" s="98" t="str" cm="1">
+      <c r="C50" s="94" t="str" cm="1">
         <f t="array" ref="C50">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattapon</v>
       </c>
-      <c r="D50" s="98" t="s">
+      <c r="D50" s="94" t="s">
         <v>704</v>
       </c>
       <c r="E50" s="27" t="s">
@@ -18883,11 +18909,11 @@
       <c r="B51" s="27" t="s">
         <v>705</v>
       </c>
-      <c r="C51" s="98" t="str" cm="1">
+      <c r="C51" s="94" t="str" cm="1">
         <f t="array" ref="C51">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattapong</v>
       </c>
-      <c r="D51" s="98" t="s">
+      <c r="D51" s="94" t="s">
         <v>706</v>
       </c>
       <c r="E51" s="27" t="s">
@@ -18907,11 +18933,11 @@
       <c r="B52" s="27" t="s">
         <v>709</v>
       </c>
-      <c r="C52" s="98" t="str" cm="1">
+      <c r="C52" s="94" t="str" cm="1">
         <f t="array" ref="C52">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattapong</v>
       </c>
-      <c r="D52" s="98" t="s">
+      <c r="D52" s="94" t="s">
         <v>710</v>
       </c>
       <c r="E52" s="27" t="s">
@@ -18931,11 +18957,11 @@
       <c r="B53" s="27" t="s">
         <v>711</v>
       </c>
-      <c r="C53" s="98" t="str" cm="1">
+      <c r="C53" s="94" t="str" cm="1">
         <f t="array" ref="C53">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nattayaporn</v>
       </c>
-      <c r="D53" s="98" t="s">
+      <c r="D53" s="94" t="s">
         <v>712</v>
       </c>
       <c r="E53" s="27" t="s">
@@ -18955,11 +18981,11 @@
       <c r="B54" s="27" t="s">
         <v>715</v>
       </c>
-      <c r="C54" s="98" t="str" cm="1">
+      <c r="C54" s="94" t="str" cm="1">
         <f t="array" ref="C54">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Natthaphong</v>
       </c>
-      <c r="D54" s="98" t="s">
+      <c r="D54" s="94" t="s">
         <v>716</v>
       </c>
       <c r="E54" s="27" t="s">
@@ -18979,11 +19005,11 @@
       <c r="B55" s="27" t="s">
         <v>717</v>
       </c>
-      <c r="C55" s="98" t="str" cm="1">
+      <c r="C55" s="94" t="str" cm="1">
         <f t="array" ref="C55">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Nichanan</v>
       </c>
-      <c r="D55" s="98" t="s">
+      <c r="D55" s="94" t="s">
         <v>718</v>
       </c>
       <c r="E55" s="27" t="s">
@@ -19003,8 +19029,8 @@
       <c r="B56" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="C56" s="98"/>
-      <c r="D56" s="98"/>
+      <c r="C56" s="94"/>
+      <c r="D56" s="94"/>
       <c r="E56" s="27"/>
       <c r="F56" s="27"/>
       <c r="G56" s="27"/>
@@ -19016,11 +19042,11 @@
       <c r="B57" s="27" t="s">
         <v>721</v>
       </c>
-      <c r="C57" s="98" t="str" cm="1">
+      <c r="C57" s="94" t="str" cm="1">
         <f t="array" ref="C57">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Onuma</v>
       </c>
-      <c r="D57" s="98" t="s">
+      <c r="D57" s="94" t="s">
         <v>722</v>
       </c>
       <c r="E57" s="27" t="s">
@@ -19040,11 +19066,11 @@
       <c r="B58" s="27" t="s">
         <v>724</v>
       </c>
-      <c r="C58" s="98" t="str" cm="1">
+      <c r="C58" s="94" t="str" cm="1">
         <f t="array" ref="C58">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pairin</v>
       </c>
-      <c r="D58" s="98" t="s">
+      <c r="D58" s="94" t="s">
         <v>725</v>
       </c>
       <c r="E58" s="27" t="s">
@@ -19064,11 +19090,11 @@
       <c r="B59" s="27" t="s">
         <v>728</v>
       </c>
-      <c r="C59" s="98" t="str" cm="1">
+      <c r="C59" s="94" t="str" cm="1">
         <f t="array" ref="C59">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pakkaporn</v>
       </c>
-      <c r="D59" s="98" t="s">
+      <c r="D59" s="94" t="s">
         <v>729</v>
       </c>
       <c r="E59" s="27" t="s">
@@ -19088,11 +19114,11 @@
       <c r="B60" s="27" t="s">
         <v>732</v>
       </c>
-      <c r="C60" s="98" t="str" cm="1">
+      <c r="C60" s="94" t="str" cm="1">
         <f t="array" ref="C60">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pakorn</v>
       </c>
-      <c r="D60" s="98" t="s">
+      <c r="D60" s="94" t="s">
         <v>733</v>
       </c>
       <c r="E60" s="27" t="s">
@@ -19112,11 +19138,11 @@
       <c r="B61" s="27" t="s">
         <v>735</v>
       </c>
-      <c r="C61" s="98" t="str" cm="1">
+      <c r="C61" s="94" t="str" cm="1">
         <f t="array" ref="C61">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pankeaw</v>
       </c>
-      <c r="D61" s="98" t="s">
+      <c r="D61" s="94" t="s">
         <v>736</v>
       </c>
       <c r="E61" s="27" t="s">
@@ -19136,11 +19162,11 @@
       <c r="B62" s="27" t="s">
         <v>738</v>
       </c>
-      <c r="C62" s="98" t="str" cm="1">
+      <c r="C62" s="94" t="str" cm="1">
         <f t="array" ref="C62">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Parata</v>
       </c>
-      <c r="D62" s="98" t="s">
+      <c r="D62" s="94" t="s">
         <v>670</v>
       </c>
       <c r="E62" s="27" t="s">
@@ -19160,11 +19186,11 @@
       <c r="B63" s="27" t="s">
         <v>739</v>
       </c>
-      <c r="C63" s="98" t="str" cm="1">
+      <c r="C63" s="94" t="str" cm="1">
         <f t="array" ref="C63">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Parichat</v>
       </c>
-      <c r="D63" s="98" t="s">
+      <c r="D63" s="94" t="s">
         <v>740</v>
       </c>
       <c r="E63" s="27" t="s">
@@ -19184,11 +19210,11 @@
       <c r="B64" s="27" t="s">
         <v>741</v>
       </c>
-      <c r="C64" s="98" t="str" cm="1">
+      <c r="C64" s="94" t="str" cm="1">
         <f t="array" ref="C64">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Parinya</v>
       </c>
-      <c r="D64" s="98" t="s">
+      <c r="D64" s="94" t="s">
         <v>742</v>
       </c>
       <c r="E64" s="27" t="s">
@@ -19208,11 +19234,11 @@
       <c r="B65" s="27" t="s">
         <v>744</v>
       </c>
-      <c r="C65" s="98" t="str" cm="1">
+      <c r="C65" s="94" t="str" cm="1">
         <f t="array" ref="C65">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Parit</v>
       </c>
-      <c r="D65" s="98" t="s">
+      <c r="D65" s="94" t="s">
         <v>745</v>
       </c>
       <c r="E65" s="27" t="s">
@@ -19232,11 +19258,11 @@
       <c r="B66" s="27" t="s">
         <v>747</v>
       </c>
-      <c r="C66" s="98" t="str" cm="1">
+      <c r="C66" s="94" t="str" cm="1">
         <f t="array" ref="C66">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Passagorn</v>
       </c>
-      <c r="D66" s="98" t="s">
+      <c r="D66" s="94" t="s">
         <v>748</v>
       </c>
       <c r="E66" s="27" t="s">
@@ -19256,11 +19282,11 @@
       <c r="B67" s="27" t="s">
         <v>750</v>
       </c>
-      <c r="C67" s="98" t="str" cm="1">
+      <c r="C67" s="94" t="str" cm="1">
         <f t="array" ref="C67">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pattama</v>
       </c>
-      <c r="D67" s="98" t="s">
+      <c r="D67" s="94" t="s">
         <v>751</v>
       </c>
       <c r="E67" s="27" t="s">
@@ -19277,14 +19303,14 @@
       <c r="A68" s="31">
         <v>66</v>
       </c>
-      <c r="B68" s="98" t="s">
+      <c r="B68" s="94" t="s">
         <v>753</v>
       </c>
-      <c r="C68" s="98" t="str" cm="1">
+      <c r="C68" s="94" t="str" cm="1">
         <f t="array" ref="C68">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Peerawut</v>
       </c>
-      <c r="D68" s="98" t="s">
+      <c r="D68" s="94" t="s">
         <v>754</v>
       </c>
       <c r="E68" s="27" t="s">
@@ -19304,11 +19330,11 @@
       <c r="B69" s="27" t="s">
         <v>755</v>
       </c>
-      <c r="C69" s="98" t="str" cm="1">
+      <c r="C69" s="94" t="str" cm="1">
         <f t="array" ref="C69">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Penthavee</v>
       </c>
-      <c r="D69" s="98" t="s">
+      <c r="D69" s="94" t="s">
         <v>756</v>
       </c>
       <c r="E69" s="27" t="s">
@@ -19328,11 +19354,11 @@
       <c r="B70" s="27" t="s">
         <v>758</v>
       </c>
-      <c r="C70" s="98" t="str" cm="1">
+      <c r="C70" s="94" t="str" cm="1">
         <f t="array" ref="C70">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Phatthanan</v>
       </c>
-      <c r="D70" s="98" t="s">
+      <c r="D70" s="94" t="s">
         <v>759</v>
       </c>
       <c r="E70" s="27" t="s">
@@ -19352,11 +19378,11 @@
       <c r="B71" s="27" t="s">
         <v>760</v>
       </c>
-      <c r="C71" s="98" t="str" cm="1">
+      <c r="C71" s="94" t="str" cm="1">
         <f t="array" ref="C71">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pittaya</v>
       </c>
-      <c r="D71" s="98" t="s">
+      <c r="D71" s="94" t="s">
         <v>761</v>
       </c>
       <c r="E71" s="27" t="s">
@@ -19376,11 +19402,11 @@
       <c r="B72" s="27" t="s">
         <v>764</v>
       </c>
-      <c r="C72" s="98" t="str" cm="1">
+      <c r="C72" s="94" t="str" cm="1">
         <f t="array" ref="C72">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Piyakorn</v>
       </c>
-      <c r="D72" s="98" t="s">
+      <c r="D72" s="94" t="s">
         <v>765</v>
       </c>
       <c r="E72" s="27" t="s">
@@ -19400,11 +19426,11 @@
       <c r="B73" s="27" t="s">
         <v>768</v>
       </c>
-      <c r="C73" s="98" t="str" cm="1">
+      <c r="C73" s="94" t="str" cm="1">
         <f t="array" ref="C73">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Piyapong</v>
       </c>
-      <c r="D73" s="98" t="s">
+      <c r="D73" s="94" t="s">
         <v>769</v>
       </c>
       <c r="E73" s="27" t="s">
@@ -19424,11 +19450,11 @@
       <c r="B74" s="27" t="s">
         <v>772</v>
       </c>
-      <c r="C74" s="98" t="str" cm="1">
+      <c r="C74" s="94" t="str" cm="1">
         <f t="array" ref="C74">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Poonkeat</v>
       </c>
-      <c r="D74" s="98" t="s">
+      <c r="D74" s="94" t="s">
         <v>773</v>
       </c>
       <c r="E74" s="27" t="s">
@@ -19448,11 +19474,11 @@
       <c r="B75" s="27" t="s">
         <v>775</v>
       </c>
-      <c r="C75" s="98" t="str" cm="1">
+      <c r="C75" s="94" t="str" cm="1">
         <f t="array" ref="C75">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pornpimon</v>
       </c>
-      <c r="D75" s="98" t="s">
+      <c r="D75" s="94" t="s">
         <v>776</v>
       </c>
       <c r="E75" s="27" t="s">
@@ -19472,11 +19498,11 @@
       <c r="B76" s="27" t="s">
         <v>779</v>
       </c>
-      <c r="C76" s="98" t="str" cm="1">
+      <c r="C76" s="94" t="str" cm="1">
         <f t="array" ref="C76">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Pracha</v>
       </c>
-      <c r="D76" s="98" t="s">
+      <c r="D76" s="94" t="s">
         <v>780</v>
       </c>
       <c r="E76" s="27" t="s">
@@ -19496,11 +19522,11 @@
       <c r="B77" s="27" t="s">
         <v>781</v>
       </c>
-      <c r="C77" s="98" t="str" cm="1">
+      <c r="C77" s="94" t="str" cm="1">
         <f t="array" ref="C77">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Prapaporn</v>
       </c>
-      <c r="D77" s="98" t="s">
+      <c r="D77" s="94" t="s">
         <v>782</v>
       </c>
       <c r="E77" s="27" t="s">
@@ -19520,11 +19546,11 @@
       <c r="B78" s="27" t="s">
         <v>784</v>
       </c>
-      <c r="C78" s="98" t="str" cm="1">
+      <c r="C78" s="94" t="str" cm="1">
         <f t="array" ref="C78">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Punyawee</v>
       </c>
-      <c r="D78" s="98" t="s">
+      <c r="D78" s="94" t="s">
         <v>785</v>
       </c>
       <c r="E78" s="27" t="s">
@@ -19544,11 +19570,11 @@
       <c r="B79" s="27" t="s">
         <v>786</v>
       </c>
-      <c r="C79" s="98" t="str" cm="1">
+      <c r="C79" s="94" t="str" cm="1">
         <f t="array" ref="C79">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Ramanee</v>
       </c>
-      <c r="D79" s="98" t="s">
+      <c r="D79" s="94" t="s">
         <v>540</v>
       </c>
       <c r="E79" s="27" t="s">
@@ -19568,11 +19594,11 @@
       <c r="B80" s="27" t="s">
         <v>787</v>
       </c>
-      <c r="C80" s="98" t="str" cm="1">
+      <c r="C80" s="94" t="str" cm="1">
         <f t="array" ref="C80">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Rath</v>
       </c>
-      <c r="D80" s="98" t="s">
+      <c r="D80" s="94" t="s">
         <v>788</v>
       </c>
       <c r="E80" s="27" t="s">
@@ -19592,11 +19618,11 @@
       <c r="B81" s="27" t="s">
         <v>790</v>
       </c>
-      <c r="C81" s="98" t="str" cm="1">
+      <c r="C81" s="94" t="str" cm="1">
         <f t="array" ref="C81">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Samart</v>
       </c>
-      <c r="D81" s="98" t="s">
+      <c r="D81" s="94" t="s">
         <v>791</v>
       </c>
       <c r="E81" s="27" t="s">
@@ -19616,11 +19642,11 @@
       <c r="B82" s="27" t="s">
         <v>792</v>
       </c>
-      <c r="C82" s="98" t="str" cm="1">
+      <c r="C82" s="94" t="str" cm="1">
         <f t="array" ref="C82">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sansren</v>
       </c>
-      <c r="D82" s="98" t="s">
+      <c r="D82" s="94" t="s">
         <v>793</v>
       </c>
       <c r="E82" s="27" t="s">
@@ -19640,11 +19666,11 @@
       <c r="B83" s="27" t="s">
         <v>794</v>
       </c>
-      <c r="C83" s="98" t="str" cm="1">
+      <c r="C83" s="94" t="str" cm="1">
         <f t="array" ref="C83">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Saranya</v>
       </c>
-      <c r="D83" s="98" t="s">
+      <c r="D83" s="94" t="s">
         <v>795</v>
       </c>
       <c r="E83" s="27" t="s">
@@ -19664,11 +19690,11 @@
       <c r="B84" s="44" t="s">
         <v>797</v>
       </c>
-      <c r="C84" s="98" t="str" cm="1">
+      <c r="C84" s="94" t="str" cm="1">
         <f t="array" ref="C84">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sarawut</v>
       </c>
-      <c r="D84" s="98" t="s">
+      <c r="D84" s="94" t="s">
         <v>798</v>
       </c>
       <c r="E84" s="27" t="s">
@@ -19688,11 +19714,11 @@
       <c r="B85" s="27" t="s">
         <v>800</v>
       </c>
-      <c r="C85" s="98" t="str" cm="1">
+      <c r="C85" s="94" t="str" cm="1">
         <f t="array" ref="C85">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sayamon</v>
       </c>
-      <c r="D85" s="98" t="s">
+      <c r="D85" s="94" t="s">
         <v>801</v>
       </c>
       <c r="E85" s="27" t="s">
@@ -19712,11 +19738,11 @@
       <c r="B86" s="27" t="s">
         <v>803</v>
       </c>
-      <c r="C86" s="98" t="str" cm="1">
+      <c r="C86" s="94" t="str" cm="1">
         <f t="array" ref="C86">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sirinapa</v>
       </c>
-      <c r="D86" s="98" t="s">
+      <c r="D86" s="94" t="s">
         <v>804</v>
       </c>
       <c r="E86" s="27" t="s">
@@ -19736,11 +19762,11 @@
       <c r="B87" s="27" t="s">
         <v>806</v>
       </c>
-      <c r="C87" s="98" t="str" cm="1">
+      <c r="C87" s="94" t="str" cm="1">
         <f t="array" ref="C87">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sirinat</v>
       </c>
-      <c r="D87" s="98" t="s">
+      <c r="D87" s="94" t="s">
         <v>807</v>
       </c>
       <c r="E87" s="27" t="s">
@@ -19760,11 +19786,11 @@
       <c r="B88" s="27" t="s">
         <v>809</v>
       </c>
-      <c r="C88" s="98" t="str" cm="1">
+      <c r="C88" s="94" t="str" cm="1">
         <f t="array" ref="C88">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Suchart</v>
       </c>
-      <c r="D88" s="98" t="s">
+      <c r="D88" s="94" t="s">
         <v>729</v>
       </c>
       <c r="E88" s="27" t="s">
@@ -19784,11 +19810,11 @@
       <c r="B89" s="27" t="s">
         <v>810</v>
       </c>
-      <c r="C89" s="98" t="str" cm="1">
+      <c r="C89" s="94" t="str" cm="1">
         <f t="array" ref="C89">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Suparchai</v>
       </c>
-      <c r="D89" s="98" t="s">
+      <c r="D89" s="94" t="s">
         <v>811</v>
       </c>
       <c r="E89" s="27" t="s">
@@ -19808,11 +19834,11 @@
       <c r="B90" s="27" t="s">
         <v>812</v>
       </c>
-      <c r="C90" s="98" t="str" cm="1">
+      <c r="C90" s="94" t="str" cm="1">
         <f t="array" ref="C90">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Supatchanikorn</v>
       </c>
-      <c r="D90" s="98" t="s">
+      <c r="D90" s="94" t="s">
         <v>813</v>
       </c>
       <c r="E90" s="27" t="s">
@@ -19832,11 +19858,11 @@
       <c r="B91" s="27" t="s">
         <v>816</v>
       </c>
-      <c r="C91" s="98" t="str" cm="1">
+      <c r="C91" s="94" t="str" cm="1">
         <f t="array" ref="C91">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sutiwat</v>
       </c>
-      <c r="D91" s="98" t="s">
+      <c r="D91" s="94" t="s">
         <v>817</v>
       </c>
       <c r="E91" s="27" t="s">
@@ -19856,11 +19882,11 @@
       <c r="B92" s="27" t="s">
         <v>820</v>
       </c>
-      <c r="C92" s="98" t="str" cm="1">
+      <c r="C92" s="94" t="str" cm="1">
         <f t="array" ref="C92">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sutthanom</v>
       </c>
-      <c r="D92" s="98" t="s">
+      <c r="D92" s="94" t="s">
         <v>602</v>
       </c>
       <c r="E92" s="27" t="s">
@@ -19880,11 +19906,11 @@
       <c r="B93" s="27" t="s">
         <v>822</v>
       </c>
-      <c r="C93" s="98" t="str" cm="1">
+      <c r="C93" s="94" t="str" cm="1">
         <f t="array" ref="C93">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Sutthipong</v>
       </c>
-      <c r="D93" s="98" t="s">
+      <c r="D93" s="94" t="s">
         <v>823</v>
       </c>
       <c r="E93" s="27" t="s">
@@ -19904,11 +19930,11 @@
       <c r="B94" s="27" t="s">
         <v>824</v>
       </c>
-      <c r="C94" s="98" t="str" cm="1">
+      <c r="C94" s="94" t="str" cm="1">
         <f t="array" ref="C94">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Suwimon</v>
       </c>
-      <c r="D94" s="98" t="s">
+      <c r="D94" s="94" t="s">
         <v>825</v>
       </c>
       <c r="E94" s="27" t="s">
@@ -19928,11 +19954,11 @@
       <c r="B95" s="27" t="s">
         <v>828</v>
       </c>
-      <c r="C95" s="98" t="str" cm="1">
+      <c r="C95" s="94" t="str" cm="1">
         <f t="array" ref="C95">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tachit</v>
       </c>
-      <c r="D95" s="98" t="s">
+      <c r="D95" s="94" t="s">
         <v>829</v>
       </c>
       <c r="E95" s="27" t="s">
@@ -19952,11 +19978,11 @@
       <c r="B96" s="27" t="s">
         <v>831</v>
       </c>
-      <c r="C96" s="98" t="str" cm="1">
+      <c r="C96" s="94" t="str" cm="1">
         <f t="array" ref="C96">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tananon</v>
       </c>
-      <c r="D96" s="98" t="s">
+      <c r="D96" s="94" t="s">
         <v>602</v>
       </c>
       <c r="E96" s="27" t="s">
@@ -19976,11 +20002,11 @@
       <c r="B97" s="27" t="s">
         <v>834</v>
       </c>
-      <c r="C97" s="98" t="str" cm="1">
+      <c r="C97" s="94" t="str" cm="1">
         <f t="array" ref="C97">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tarika</v>
       </c>
-      <c r="D97" s="98" t="s">
+      <c r="D97" s="94" t="s">
         <v>835</v>
       </c>
       <c r="E97" s="27" t="s">
@@ -20000,11 +20026,11 @@
       <c r="B98" s="27" t="s">
         <v>837</v>
       </c>
-      <c r="C98" s="98" t="str" cm="1">
+      <c r="C98" s="94" t="str" cm="1">
         <f t="array" ref="C98">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tawan</v>
       </c>
-      <c r="D98" s="98" t="s">
+      <c r="D98" s="94" t="s">
         <v>838</v>
       </c>
       <c r="E98" s="27" t="s">
@@ -20024,11 +20050,11 @@
       <c r="B99" s="27" t="s">
         <v>841</v>
       </c>
-      <c r="C99" s="98" t="str" cm="1">
+      <c r="C99" s="94" t="str" cm="1">
         <f t="array" ref="C99">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Teerapong</v>
       </c>
-      <c r="D99" s="98" t="s">
+      <c r="D99" s="94" t="s">
         <v>842</v>
       </c>
       <c r="E99" s="27" t="s">
@@ -20048,11 +20074,11 @@
       <c r="B100" s="27" t="s">
         <v>843</v>
       </c>
-      <c r="C100" s="98" t="str" cm="1">
+      <c r="C100" s="94" t="str" cm="1">
         <f t="array" ref="C100">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Teraphich</v>
       </c>
-      <c r="D100" s="98" t="s">
+      <c r="D100" s="94" t="s">
         <v>844</v>
       </c>
       <c r="E100" s="27" t="s">
@@ -20072,11 +20098,11 @@
       <c r="B101" s="27" t="s">
         <v>845</v>
       </c>
-      <c r="C101" s="98" t="str" cm="1">
+      <c r="C101" s="94" t="str" cm="1">
         <f t="array" ref="C101">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Terdkiet</v>
       </c>
-      <c r="D101" s="98" t="s">
+      <c r="D101" s="94" t="s">
         <v>846</v>
       </c>
       <c r="E101" s="27" t="s">
@@ -20096,11 +20122,11 @@
       <c r="B102" s="27" t="s">
         <v>847</v>
       </c>
-      <c r="C102" s="98" t="str" cm="1">
+      <c r="C102" s="94" t="str" cm="1">
         <f t="array" ref="C102">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tewara</v>
       </c>
-      <c r="D102" s="98" t="s">
+      <c r="D102" s="94" t="s">
         <v>848</v>
       </c>
       <c r="E102" s="27" t="s">
@@ -20120,11 +20146,11 @@
       <c r="B103" s="27" t="s">
         <v>850</v>
       </c>
-      <c r="C103" s="98" t="str" cm="1">
+      <c r="C103" s="94" t="str" cm="1">
         <f t="array" ref="C103">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Thananrath</v>
       </c>
-      <c r="D103" s="98" t="s">
+      <c r="D103" s="94" t="s">
         <v>851</v>
       </c>
       <c r="E103" s="27" t="s">
@@ -20144,11 +20170,11 @@
       <c r="B104" s="27" t="s">
         <v>852</v>
       </c>
-      <c r="C104" s="98" t="str" cm="1">
+      <c r="C104" s="94" t="str" cm="1">
         <f t="array" ref="C104">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Thanyapong</v>
       </c>
-      <c r="D104" s="98" t="s">
+      <c r="D104" s="94" t="s">
         <v>853</v>
       </c>
       <c r="E104" s="27" t="s">
@@ -20168,11 +20194,11 @@
       <c r="B105" s="27" t="s">
         <v>854</v>
       </c>
-      <c r="C105" s="98" t="str" cm="1">
+      <c r="C105" s="94" t="str" cm="1">
         <f t="array" ref="C105">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Thummapradit</v>
       </c>
-      <c r="D105" s="98" t="s">
+      <c r="D105" s="94" t="s">
         <v>855</v>
       </c>
       <c r="E105" s="27" t="s">
@@ -20192,11 +20218,11 @@
       <c r="B106" s="27" t="s">
         <v>856</v>
       </c>
-      <c r="C106" s="98" t="str" cm="1">
+      <c r="C106" s="94" t="str" cm="1">
         <f t="array" ref="C106">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tuansuhaimin</v>
       </c>
-      <c r="D106" s="98" t="s">
+      <c r="D106" s="94" t="s">
         <v>857</v>
       </c>
       <c r="E106" s="27" t="s">
@@ -20216,14 +20242,14 @@
       <c r="B107" s="27" t="s">
         <v>858</v>
       </c>
-      <c r="C107" s="98" t="str" cm="1">
+      <c r="C107" s="94" t="str" cm="1">
         <f t="array" ref="C107">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Tun</v>
       </c>
-      <c r="D107" s="98" t="s">
+      <c r="D107" s="94" t="s">
         <v>859</v>
       </c>
-      <c r="E107" s="102" t="s">
+      <c r="E107" s="98" t="s">
         <v>330</v>
       </c>
       <c r="F107" s="27" t="s">
@@ -20240,11 +20266,11 @@
       <c r="B108" s="27" t="s">
         <v>860</v>
       </c>
-      <c r="C108" s="98" t="str" cm="1">
+      <c r="C108" s="94" t="str" cm="1">
         <f t="array" ref="C108">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Uthai</v>
       </c>
-      <c r="D108" s="98" t="s">
+      <c r="D108" s="94" t="s">
         <v>861</v>
       </c>
       <c r="E108" s="27" t="s">
@@ -20264,11 +20290,11 @@
       <c r="B109" s="27" t="s">
         <v>862</v>
       </c>
-      <c r="C109" s="98" t="str" cm="1">
+      <c r="C109" s="94" t="str" cm="1">
         <f t="array" ref="C109">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Utit</v>
       </c>
-      <c r="D109" s="98" t="s">
+      <c r="D109" s="94" t="s">
         <v>863</v>
       </c>
       <c r="E109" s="27" t="s">
@@ -20288,11 +20314,11 @@
       <c r="B110" s="27" t="s">
         <v>864</v>
       </c>
-      <c r="C110" s="98" t="str" cm="1">
+      <c r="C110" s="94" t="str" cm="1">
         <f t="array" ref="C110">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Wanna</v>
       </c>
-      <c r="D110" s="98" t="s">
+      <c r="D110" s="94" t="s">
         <v>865</v>
       </c>
       <c r="E110" s="27" t="s">
@@ -20312,11 +20338,11 @@
       <c r="B111" s="27" t="s">
         <v>866</v>
       </c>
-      <c r="C111" s="98" t="str" cm="1">
+      <c r="C111" s="94" t="str" cm="1">
         <f t="array" ref="C111">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Wassaris</v>
       </c>
-      <c r="D111" s="98" t="s">
+      <c r="D111" s="94" t="s">
         <v>867</v>
       </c>
       <c r="E111" s="27" t="s">
@@ -20336,11 +20362,11 @@
       <c r="B112" s="27" t="s">
         <v>868</v>
       </c>
-      <c r="C112" s="98" t="str" cm="1">
+      <c r="C112" s="94" t="str" cm="1">
         <f t="array" ref="C112">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Watcharapol</v>
       </c>
-      <c r="D112" s="98" t="s">
+      <c r="D112" s="94" t="s">
         <v>869</v>
       </c>
       <c r="E112" s="27" t="s">
@@ -20360,11 +20386,11 @@
       <c r="B113" s="27" t="s">
         <v>872</v>
       </c>
-      <c r="C113" s="98" t="str" cm="1">
+      <c r="C113" s="94" t="str" cm="1">
         <f t="array" ref="C113">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Watcharee</v>
       </c>
-      <c r="D113" s="98" t="s">
+      <c r="D113" s="94" t="s">
         <v>873</v>
       </c>
       <c r="E113" s="27" t="s">
@@ -20384,11 +20410,11 @@
       <c r="B114" s="27" t="s">
         <v>875</v>
       </c>
-      <c r="C114" s="98" t="str" cm="1">
+      <c r="C114" s="94" t="str" cm="1">
         <f t="array" ref="C114">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Watcharin</v>
       </c>
-      <c r="D114" s="98" t="s">
+      <c r="D114" s="94" t="s">
         <v>876</v>
       </c>
       <c r="E114" s="27" t="s">
@@ -20408,11 +20434,11 @@
       <c r="B115" s="27" t="s">
         <v>878</v>
       </c>
-      <c r="C115" s="98" t="str" cm="1">
+      <c r="C115" s="94" t="str" cm="1">
         <f t="array" ref="C115">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Wirat</v>
       </c>
-      <c r="D115" s="98" t="s">
+      <c r="D115" s="94" t="s">
         <v>879</v>
       </c>
       <c r="E115" s="27" t="s">
@@ -20432,11 +20458,11 @@
       <c r="B116" s="27" t="s">
         <v>881</v>
       </c>
-      <c r="C116" s="98" t="str" cm="1">
+      <c r="C116" s="94" t="str" cm="1">
         <f t="array" ref="C116">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Wiriya</v>
       </c>
-      <c r="D116" s="98" t="s">
+      <c r="D116" s="94" t="s">
         <v>882</v>
       </c>
       <c r="E116" s="27" t="s">
@@ -20456,11 +20482,11 @@
       <c r="B117" s="27" t="s">
         <v>884</v>
       </c>
-      <c r="C117" s="98" t="str" cm="1">
+      <c r="C117" s="94" t="str" cm="1">
         <f t="array" ref="C117">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Witchuda</v>
       </c>
-      <c r="D117" s="98" t="s">
+      <c r="D117" s="94" t="s">
         <v>885</v>
       </c>
       <c r="E117" s="27" t="s">
@@ -20480,11 +20506,11 @@
       <c r="B118" s="27" t="s">
         <v>886</v>
       </c>
-      <c r="C118" s="98" t="str" cm="1">
+      <c r="C118" s="94" t="str" cm="1">
         <f t="array" ref="C118">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Woranan</v>
       </c>
-      <c r="D118" s="98" t="s">
+      <c r="D118" s="94" t="s">
         <v>887</v>
       </c>
       <c r="E118" s="27" t="s">
@@ -20504,11 +20530,11 @@
       <c r="B119" s="27" t="s">
         <v>888</v>
       </c>
-      <c r="C119" s="98" t="str" cm="1">
+      <c r="C119" s="94" t="str" cm="1">
         <f t="array" ref="C119">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Worawit</v>
       </c>
-      <c r="D119" s="98" t="s">
+      <c r="D119" s="94" t="s">
         <v>889</v>
       </c>
       <c r="E119" s="27" t="s">
@@ -20528,11 +20554,11 @@
       <c r="B120" s="27" t="s">
         <v>892</v>
       </c>
-      <c r="C120" s="98" t="str" cm="1">
+      <c r="C120" s="94" t="str" cm="1">
         <f t="array" ref="C120">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Yongyoot</v>
       </c>
-      <c r="D120" s="98" t="s">
+      <c r="D120" s="94" t="s">
         <v>893</v>
       </c>
       <c r="E120" s="27" t="s">
@@ -20552,11 +20578,11 @@
       <c r="B121" s="27" t="s">
         <v>894</v>
       </c>
-      <c r="C121" s="98" t="str" cm="1">
+      <c r="C121" s="94" t="str" cm="1">
         <f t="array" ref="C121">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Yossawadee</v>
       </c>
-      <c r="D121" s="98" t="s">
+      <c r="D121" s="94" t="s">
         <v>895</v>
       </c>
       <c r="E121" s="27" t="s">
@@ -20576,11 +20602,11 @@
       <c r="B122" s="27" t="s">
         <v>898</v>
       </c>
-      <c r="C122" s="98" t="e" cm="1">
+      <c r="C122" s="94" t="e" cm="1">
         <f t="array" ref="C122">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>#REF!</v>
       </c>
-      <c r="D122" s="98" t="s">
+      <c r="D122" s="94" t="s">
         <v>899</v>
       </c>
       <c r="E122" s="27" t="s">
@@ -20600,14 +20626,14 @@
       <c r="B123" s="27" t="s">
         <v>902</v>
       </c>
-      <c r="C123" s="98" t="str" cm="1">
+      <c r="C123" s="94" t="str" cm="1">
         <f t="array" ref="C123">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Chanin</v>
       </c>
-      <c r="D123" s="98" t="s">
+      <c r="D123" s="94" t="s">
         <v>903</v>
       </c>
-      <c r="E123" s="103" t="s">
+      <c r="E123" s="99" t="s">
         <v>904</v>
       </c>
       <c r="F123" s="27" t="s">
@@ -20624,14 +20650,14 @@
       <c r="B124" s="1" t="s">
         <v>905</v>
       </c>
-      <c r="C124" s="98" t="str" cm="1">
+      <c r="C124" s="94" t="str" cm="1">
         <f t="array" ref="C124">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Hataurat</v>
       </c>
-      <c r="D124" s="98" t="s">
+      <c r="D124" s="94" t="s">
         <v>906</v>
       </c>
-      <c r="E124" s="103" t="s">
+      <c r="E124" s="99" t="s">
         <v>907</v>
       </c>
       <c r="F124" s="1" t="s">
@@ -20648,14 +20674,14 @@
       <c r="B125" s="1" t="s">
         <v>909</v>
       </c>
-      <c r="C125" s="98" t="str" cm="1">
+      <c r="C125" s="94" t="str" cm="1">
         <f t="array" ref="C125">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>Ismail</v>
       </c>
-      <c r="D125" s="98" t="s">
+      <c r="D125" s="94" t="s">
         <v>910</v>
       </c>
-      <c r="E125" s="103" t="s">
+      <c r="E125" s="99" t="s">
         <v>911</v>
       </c>
       <c r="F125" s="1" t="s">
@@ -20672,11 +20698,11 @@
       <c r="B126" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C126" s="98" t="e" cm="1">
+      <c r="C126" s="94" t="e" cm="1">
         <f t="array" ref="C126">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>#REF!</v>
       </c>
-      <c r="D126" s="98"/>
+      <c r="D126" s="94"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.65">
       <c r="A127" s="31">
@@ -20685,11 +20711,11 @@
       <c r="B127" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C127" s="98" t="e" cm="1">
+      <c r="C127" s="94" t="e" cm="1">
         <f t="array" ref="C127">INDEX(_xlfn.TEXTSPLIT(Table14[[#This Row],[Display name]], " "), 2)</f>
         <v>#REF!</v>
       </c>
-      <c r="D127" s="98"/>
+      <c r="D127" s="94"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.65">
       <c r="A128" s="126" t="s">
@@ -21004,6 +21030,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c5a18c76-b749-4343-9c1d-303eadb79e6c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f6a3cb3-7ed8-4dff-adae-eea786e7335c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F5C62EC7A8419A449F9B86172F15A377" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b7baa5e68384fa41840c04eb28526fc0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1f6a3cb3-7ed8-4dff-adae-eea786e7335c" xmlns:ns3="c5a18c76-b749-4343-9c1d-303eadb79e6c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e64537676c8af67489fbedd0d2d3ecad" ns2:_="" ns3:_="">
     <xsd:import namespace="1f6a3cb3-7ed8-4dff-adae-eea786e7335c"/>
@@ -21232,27 +21278,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c5a18c76-b749-4343-9c1d-303eadb79e6c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1f6a3cb3-7ed8-4dff-adae-eea786e7335c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{494642E4-5891-4D31-A5AC-FC3276A27EF8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c5a18c76-b749-4343-9c1d-303eadb79e6c"/>
+    <ds:schemaRef ds:uri="1f6a3cb3-7ed8-4dff-adae-eea786e7335c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AFFBEF8-2963-423F-BE2B-F84A2662949F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD5BBDA0-F671-41E3-A46A-8B76EAB5ECC1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21269,23 +21314,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{494642E4-5891-4D31-A5AC-FC3276A27EF8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c5a18c76-b749-4343-9c1d-303eadb79e6c"/>
-    <ds:schemaRef ds:uri="1f6a3cb3-7ed8-4dff-adae-eea786e7335c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AFFBEF8-2963-423F-BE2B-F84A2662949F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>